<commit_message>
female pair auctions: pair bidding UI, 20k pair base price, roster updates & renumbered male IDs
</commit_message>
<xml_diff>
--- a/CLASS 12TH PLAYER (1).xlsx
+++ b/CLASS 12TH PLAYER (1).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aaradhya-rai/EHPL-Auctions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_50945E3DD4863F03D0A6C16E4F13BC1E65949CAD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2FBBD7C-D20F-6E48-9E6E-9B60A7DACAAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4420" yWindow="660" windowWidth="13400" windowHeight="17360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet5" sheetId="1" r:id="rId1"/>
@@ -36,137 +36,62 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="89">
   <si>
     <t>NAME</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTIVITY </t>
-  </si>
-  <si>
-    <t>PREVIOUS TEAM</t>
-  </si>
-  <si>
     <t>AARADHYA RAI</t>
   </si>
   <si>
-    <t>WALL CLIMBING</t>
-  </si>
-  <si>
-    <t>DHRUVA</t>
-  </si>
-  <si>
     <t>AKSHIT SHARMA</t>
   </si>
   <si>
-    <t>FOOTBALL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">YODHA </t>
-  </si>
-  <si>
     <t>AARADHYA GARG</t>
   </si>
   <si>
-    <t>BASKETBALL</t>
-  </si>
-  <si>
-    <t>NA</t>
-  </si>
-  <si>
     <t>ARYAMAN GARG</t>
   </si>
   <si>
-    <t>RANBHOOMI</t>
-  </si>
-  <si>
     <t xml:space="preserve">KARTIK CHAUDHARY </t>
   </si>
   <si>
-    <t>THROWBALL</t>
-  </si>
-  <si>
-    <t>AGNIASTRA</t>
-  </si>
-  <si>
     <t xml:space="preserve">KAVYA JAIN </t>
   </si>
   <si>
-    <t>KSHATRIYA</t>
-  </si>
-  <si>
     <t>NILESH AGRAWAL</t>
   </si>
   <si>
-    <t>TABLE TENNIS</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
     <t>SWAYAM BHERWANI</t>
   </si>
   <si>
-    <t>BADMINTON</t>
-  </si>
-  <si>
-    <t>CHAKRAVYU</t>
-  </si>
-  <si>
     <t xml:space="preserve">YASHMANYA RATHI </t>
   </si>
   <si>
-    <t xml:space="preserve">CRICKET </t>
-  </si>
-  <si>
-    <t>KURUKSHETRA</t>
-  </si>
-  <si>
     <t xml:space="preserve">OJASVA GUPTA </t>
   </si>
   <si>
-    <t xml:space="preserve">ATHELETICS </t>
-  </si>
-  <si>
-    <t>TRISHUL</t>
-  </si>
-  <si>
     <t>PUNEET KHEMKA</t>
   </si>
   <si>
-    <t>MARTIAL ARTS</t>
-  </si>
-  <si>
     <t>RANBHOOMIVEER SINGH SISODIYA</t>
   </si>
   <si>
-    <t>SHOORVEER</t>
-  </si>
-  <si>
     <t>SANJAN GAUR</t>
   </si>
   <si>
     <t xml:space="preserve">VARCHASAV JAIN </t>
   </si>
   <si>
-    <t>SQUASH</t>
-  </si>
-  <si>
     <t>RUDRAKSH JAJAWARA</t>
   </si>
   <si>
-    <t>RAJ</t>
-  </si>
-  <si>
     <t>ANSHUMAN AGRAWAL</t>
   </si>
   <si>
     <t xml:space="preserve">ARPIT AGRAWAL </t>
   </si>
   <si>
-    <t>TEAKWONDO</t>
-  </si>
-  <si>
     <t xml:space="preserve">DEWANK AILANI </t>
   </si>
   <si>
@@ -179,51 +104,30 @@
     <t xml:space="preserve">SHRISH BAJAJ </t>
   </si>
   <si>
-    <t>HANDBALL</t>
-  </si>
-  <si>
     <t>SOUMYA AGRAWAL</t>
   </si>
   <si>
-    <t>JUDO</t>
-  </si>
-  <si>
     <t xml:space="preserve">ANSHUMAN SINGH </t>
   </si>
   <si>
     <t>ARNAV AGRAWAL</t>
   </si>
   <si>
-    <t>TAEKWONDO</t>
-  </si>
-  <si>
-    <t>SAMRAT</t>
-  </si>
-  <si>
     <t>HEMANT VARYANI</t>
   </si>
   <si>
     <t xml:space="preserve">ISHIT MANKANI </t>
   </si>
   <si>
-    <t>NETBALL</t>
-  </si>
-  <si>
     <t xml:space="preserve">KALP TALREJA </t>
   </si>
   <si>
     <t>KUSHAGRA JAIN</t>
   </si>
   <si>
-    <t>RAJTANTRA</t>
-  </si>
-  <si>
     <t>MANTRA TANEJA</t>
   </si>
   <si>
-    <t>HOCKEY</t>
-  </si>
-  <si>
     <t>PARSAV JAIN</t>
   </si>
   <si>
@@ -233,9 +137,6 @@
     <t>PRADYUMAN AGRAWAL</t>
   </si>
   <si>
-    <t xml:space="preserve">BRAMASTRA </t>
-  </si>
-  <si>
     <t>LAKSHYAJEET SINGH CHOUHAN</t>
   </si>
   <si>
@@ -254,36 +155,18 @@
     <t xml:space="preserve">RAUNAK AGRAWAL </t>
   </si>
   <si>
-    <t>ATHELETICS</t>
-  </si>
-  <si>
     <t xml:space="preserve">RISHIT GUPTA </t>
   </si>
   <si>
-    <t>CHESS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RUDRANBHOOMISH  AGRAWAL </t>
-  </si>
-  <si>
-    <t>AGNIASTRAASTRA</t>
-  </si>
-  <si>
     <t>RUTRAJ JAIN</t>
   </si>
   <si>
-    <t xml:space="preserve">MUSIC </t>
-  </si>
-  <si>
     <t xml:space="preserve">SAMARTH GARG </t>
   </si>
   <si>
     <t>SHOURYA KEDIA</t>
   </si>
   <si>
-    <t xml:space="preserve">TAEKWONDO </t>
-  </si>
-  <si>
     <t xml:space="preserve">VYOM CHANDAK </t>
   </si>
   <si>
@@ -296,15 +179,9 @@
     <t xml:space="preserve">ADITYA SACHIN AGRAWAL </t>
   </si>
   <si>
-    <t xml:space="preserve">GOLF </t>
-  </si>
-  <si>
     <t xml:space="preserve">DAKSHDITYA SINGH JHALA </t>
   </si>
   <si>
-    <t xml:space="preserve">JUDO </t>
-  </si>
-  <si>
     <t xml:space="preserve">IKSHIT AGRAWAL </t>
   </si>
   <si>
@@ -323,24 +200,12 @@
     <t xml:space="preserve">SIDDHAM NANDECHA </t>
   </si>
   <si>
-    <t xml:space="preserve">TENNIS </t>
-  </si>
-  <si>
     <t xml:space="preserve">SYED AATIF HUSSAIN </t>
   </si>
   <si>
-    <t xml:space="preserve">SQUASH </t>
-  </si>
-  <si>
-    <t>RANBHOOMIBHOOMI</t>
-  </si>
-  <si>
     <t xml:space="preserve">AARAV JAIN </t>
   </si>
   <si>
-    <t xml:space="preserve">ATHLETICS </t>
-  </si>
-  <si>
     <t xml:space="preserve">ARTH AGRAWAL </t>
   </si>
   <si>
@@ -350,21 +215,12 @@
     <t xml:space="preserve">MUDIT MAHAJAN </t>
   </si>
   <si>
-    <t xml:space="preserve">HANDBALL </t>
-  </si>
-  <si>
     <t xml:space="preserve">PARV AGRAWAL </t>
   </si>
   <si>
-    <t xml:space="preserve">TABLE TENNIS </t>
-  </si>
-  <si>
     <t xml:space="preserve">MANAS SONI </t>
   </si>
   <si>
-    <t xml:space="preserve">FOOTBALL </t>
-  </si>
-  <si>
     <t xml:space="preserve">SANSKAR JAIN </t>
   </si>
   <si>
@@ -377,9 +233,6 @@
     <t xml:space="preserve">YUVRAJ AGRAWAL </t>
   </si>
   <si>
-    <t xml:space="preserve">THROWBALL </t>
-  </si>
-  <si>
     <t>AADARSH AGRAWAL</t>
   </si>
   <si>
@@ -392,9 +245,6 @@
     <t xml:space="preserve">KESHAV SOMANI </t>
   </si>
   <si>
-    <t xml:space="preserve">VOLLEYBALL </t>
-  </si>
-  <si>
     <t xml:space="preserve">RAGHAV PATIDAR </t>
   </si>
   <si>
@@ -405,6 +255,54 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>ENTRY SONGS</t>
+  </si>
+  <si>
+    <t>Farebi</t>
+  </si>
+  <si>
+    <t>saas gali deve</t>
+  </si>
+  <si>
+    <t>Choudhar jaat ki</t>
+  </si>
+  <si>
+    <t>pehle lalkare naal</t>
+  </si>
+  <si>
+    <t>fluffing a duck</t>
+  </si>
+  <si>
+    <t>s.id.h.u</t>
+  </si>
+  <si>
+    <t>macarena</t>
+  </si>
+  <si>
+    <t>hind ke sitare</t>
+  </si>
+  <si>
+    <t>wavy</t>
+  </si>
+  <si>
+    <t>robo boy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RUDRANSH  AGRAWAL </t>
+  </si>
+  <si>
+    <t>bezuba kabse</t>
+  </si>
+  <si>
+    <t>old town road</t>
+  </si>
+  <si>
+    <t>russian bandana</t>
+  </si>
+  <si>
+    <t>thai</t>
   </si>
 </sst>
 </file>
@@ -452,10 +350,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -688,807 +587,547 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="C1" s="1"/>
     </row>
     <row r="2" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>5</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
     </row>
     <row r="3" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="2" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>8</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="C3" s="2"/>
     </row>
     <row r="4" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="2" t="s">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>11</v>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="C4" s="2"/>
     </row>
     <row r="5" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>13</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
     </row>
     <row r="6" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>16</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
     </row>
     <row r="7" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>18</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
     </row>
     <row r="8" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="2" t="s">
-        <v>19</v>
+        <v>46</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="C8" s="2"/>
     </row>
     <row r="9" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>24</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
     </row>
     <row r="10" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>27</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
     </row>
     <row r="11" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>30</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
     </row>
     <row r="12" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
     </row>
     <row r="13" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>34</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
     </row>
     <row r="14" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>34</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
     </row>
     <row r="15" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
     </row>
     <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>39</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
     </row>
     <row r="17" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
     </row>
     <row r="18" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
     </row>
     <row r="19" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
     </row>
     <row r="20" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>13</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
     </row>
     <row r="21" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
     </row>
     <row r="22" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
     </row>
     <row r="23" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>21</v>
-      </c>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
     </row>
     <row r="24" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="2" t="s">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>8</v>
-      </c>
+        <v>81</v>
+      </c>
+      <c r="C24" s="2"/>
     </row>
     <row r="25" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>53</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
     </row>
     <row r="26" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="2" t="s">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>5</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="C26" s="2"/>
     </row>
     <row r="27" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="2" t="s">
-        <v>55</v>
+        <v>6</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>8</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="C27" s="2"/>
     </row>
     <row r="28" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
     </row>
     <row r="29" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>59</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
     </row>
     <row r="30" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="B30" s="2"/>
+      <c r="C30" s="2"/>
     </row>
     <row r="31" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
     </row>
     <row r="32" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>30</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
     </row>
     <row r="33" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>65</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
     </row>
     <row r="34" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>27</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="B34" s="2"/>
+      <c r="C34" s="2"/>
     </row>
     <row r="35" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>65</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="B35" s="2"/>
+      <c r="C35" s="2"/>
     </row>
     <row r="36" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A36" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>34</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="B36" s="3">
+        <v>0.16597222222222222</v>
+      </c>
+      <c r="C36" s="2"/>
     </row>
     <row r="37" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>53</v>
-      </c>
+        <v>49</v>
+      </c>
+      <c r="B37" s="2"/>
+      <c r="C37" s="2"/>
     </row>
     <row r="38" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A38" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>18</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
     </row>
     <row r="39" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A39" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
     </row>
     <row r="40" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A40" s="2" t="s">
-        <v>73</v>
+        <v>31</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>59</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="C40" s="2"/>
     </row>
     <row r="41" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A41" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>76</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
     </row>
     <row r="42" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A42" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>76</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="B42" s="2"/>
+      <c r="C42" s="2"/>
     </row>
     <row r="43" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A43" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>53</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="B43" s="2"/>
+      <c r="C43" s="2"/>
     </row>
     <row r="44" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A44" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>69</v>
+      </c>
+      <c r="B44" s="2"/>
+      <c r="C44" s="2"/>
     </row>
     <row r="45" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A45" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>53</v>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="B45" s="2"/>
+      <c r="C45" s="2"/>
     </row>
     <row r="46" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A46" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="B46" s="2"/>
+      <c r="C46" s="2"/>
     </row>
     <row r="47" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A47" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
     </row>
     <row r="48" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A48" s="2" t="s">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>5</v>
-      </c>
+        <v>83</v>
+      </c>
+      <c r="C48" s="2"/>
     </row>
     <row r="49" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A49" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>5</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="B49" s="2"/>
+      <c r="C49" s="2"/>
     </row>
     <row r="50" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A50" s="2" t="s">
-        <v>89</v>
+        <v>15</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>8</v>
-      </c>
+        <v>85</v>
+      </c>
+      <c r="C50" s="2"/>
     </row>
     <row r="51" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A51" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>59</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="B51" s="2"/>
+      <c r="C51" s="2"/>
     </row>
     <row r="52" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A52" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="B52" s="2"/>
+      <c r="C52" s="2"/>
     </row>
     <row r="53" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A53" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="B53" s="2"/>
+      <c r="C53" s="2"/>
     </row>
     <row r="54" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A54" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>59</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="B54" s="2"/>
+      <c r="C54" s="2"/>
     </row>
     <row r="55" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A55" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>34</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="B55" s="2"/>
+      <c r="C55" s="2"/>
     </row>
     <row r="56" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A56" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B56" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>98</v>
-      </c>
+        <v>61</v>
+      </c>
+      <c r="B56" s="2"/>
+      <c r="C56" s="2"/>
     </row>
     <row r="57" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A57" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>8</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="B57" s="2"/>
+      <c r="C57" s="2"/>
     </row>
     <row r="58" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A58" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="B58" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>27</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="B58" s="2"/>
+      <c r="C58" s="2"/>
     </row>
     <row r="59" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A59" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="B59" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>76</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="B59" s="2"/>
+      <c r="C59" s="2"/>
     </row>
     <row r="60" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A60" s="2" t="s">
-        <v>103</v>
+        <v>53</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>53</v>
-      </c>
+        <v>79</v>
+      </c>
+      <c r="C60" s="2"/>
     </row>
     <row r="61" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A61" s="2" t="s">
-        <v>105</v>
+        <v>22</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="C61" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="C61" s="2"/>
     </row>
     <row r="62" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A62" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="B62" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="C62" s="2" t="s">
-        <v>76</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="B62" s="2"/>
+      <c r="C62" s="2"/>
     </row>
     <row r="63" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A63" s="2" t="s">
-        <v>109</v>
+        <v>54</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C63" s="2" t="s">
-        <v>98</v>
-      </c>
+        <v>80</v>
+      </c>
+      <c r="C63" s="2"/>
     </row>
     <row r="64" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A64" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="B64" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="C64" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="B64" s="2"/>
+      <c r="C64" s="2"/>
     </row>
     <row r="65" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A65" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="C65" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="B65" s="2"/>
+      <c r="C65" s="2"/>
     </row>
     <row r="66" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A66" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="B66" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="C66" s="2" t="s">
-        <v>27</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="B66" s="2"/>
+      <c r="C66" s="2"/>
     </row>
     <row r="67" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A67" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="B67" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="C67" s="2" t="s">
-        <v>59</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="B67" s="2"/>
+      <c r="C67" s="2"/>
     </row>
     <row r="68" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A68" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="B68" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="C68" s="2" t="s">
-        <v>98</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="B68" s="2"/>
+      <c r="C68" s="2"/>
     </row>
     <row r="69" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A69" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="B69" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="C69" s="2" t="s">
-        <v>53</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="B69" s="2"/>
+      <c r="C69" s="2"/>
     </row>
     <row r="70" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A70" s="2" t="s">
-        <v>117</v>
+        <v>9</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="C70" s="2" t="s">
-        <v>18</v>
-      </c>
+        <v>86</v>
+      </c>
+      <c r="C70" s="2"/>
     </row>
     <row r="71" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A71" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="B71" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C71" s="2" t="s">
-        <v>53</v>
-      </c>
+        <v>63</v>
+      </c>
+      <c r="B71" s="2"/>
+      <c r="C71" s="2"/>
     </row>
     <row r="72" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A72" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="B72" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C72" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="B72" s="2"/>
+      <c r="C72" s="2"/>
     </row>
     <row r="73" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A73" s="2" t="s">
-        <v>121</v>
+        <v>64</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C73" s="2" t="s">
-        <v>34</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="C73" s="2"/>
     </row>
     <row r="74" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="C74" s="2" t="s">
-        <v>122</v>
+        <v>72</v>
       </c>
     </row>
     <row r="75" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
@@ -2418,6 +2057,9 @@
     <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:A73">
+    <sortCondition ref="A2:A73"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add Team Teachers view: live display, dropdown pairing with instant sync
</commit_message>
<xml_diff>
--- a/CLASS 12TH PLAYER (1).xlsx
+++ b/CLASS 12TH PLAYER (1).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aaradhya-rai/EHPL-Auctions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2FBBD7C-D20F-6E48-9E6E-9B60A7DACAAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A327E55-9082-4446-B66A-6A6D8F4FFEA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4420" yWindow="660" windowWidth="13400" windowHeight="17360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet5" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="151">
   <si>
     <t>NAME</t>
   </si>
@@ -74,9 +74,6 @@
     <t>PUNEET KHEMKA</t>
   </si>
   <si>
-    <t>RANBHOOMIVEER SINGH SISODIYA</t>
-  </si>
-  <si>
     <t>SANJAN GAUR</t>
   </si>
   <si>
@@ -266,18 +263,9 @@
     <t>saas gali deve</t>
   </si>
   <si>
-    <t>Choudhar jaat ki</t>
-  </si>
-  <si>
-    <t>pehle lalkare naal</t>
-  </si>
-  <si>
     <t>fluffing a duck</t>
   </si>
   <si>
-    <t>s.id.h.u</t>
-  </si>
-  <si>
     <t>macarena</t>
   </si>
   <si>
@@ -287,9 +275,6 @@
     <t>wavy</t>
   </si>
   <si>
-    <t>robo boy</t>
-  </si>
-  <si>
     <t xml:space="preserve">RUDRANSH  AGRAWAL </t>
   </si>
   <si>
@@ -302,14 +287,215 @@
     <t>russian bandana</t>
   </si>
   <si>
-    <t>thai</t>
+    <t>lutt le gaya</t>
+  </si>
+  <si>
+    <t>cupid</t>
+  </si>
+  <si>
+    <t>nam deng nam som</t>
+  </si>
+  <si>
+    <t>we on go</t>
+  </si>
+  <si>
+    <t>kk da</t>
+  </si>
+  <si>
+    <t>dvorak polka</t>
+  </si>
+  <si>
+    <t>dame tu cosita</t>
+  </si>
+  <si>
+    <t>singham</t>
+  </si>
+  <si>
+    <t>RANVEER SINGH SISODIYA</t>
+  </si>
+  <si>
+    <t>4 raws</t>
+  </si>
+  <si>
+    <t>boom shaka</t>
+  </si>
+  <si>
+    <t>you talkin to me</t>
+  </si>
+  <si>
+    <t xml:space="preserve">what we do </t>
+  </si>
+  <si>
+    <t>aurea carmina</t>
+  </si>
+  <si>
+    <t>super polka</t>
+  </si>
+  <si>
+    <t>badshah o badshah 1:13</t>
+  </si>
+  <si>
+    <t>pagannini</t>
+  </si>
+  <si>
+    <t>haryane ka jaat</t>
+  </si>
+  <si>
+    <t>bink's sake</t>
+  </si>
+  <si>
+    <t>raftarrein</t>
+  </si>
+  <si>
+    <t>sultan</t>
+  </si>
+  <si>
+    <t>deadly zone</t>
+  </si>
+  <si>
+    <t>the ghost</t>
+  </si>
+  <si>
+    <t>magenta riddim 0:12</t>
+  </si>
+  <si>
+    <t>JIYA JAIN</t>
+  </si>
+  <si>
+    <t>JIYA LILANI</t>
+  </si>
+  <si>
+    <t>SIDDHI PATEL</t>
+  </si>
+  <si>
+    <t>SIDDHI PEPER</t>
+  </si>
+  <si>
+    <t>AKSHARA</t>
+  </si>
+  <si>
+    <t>APEKSHA</t>
+  </si>
+  <si>
+    <t>ANUSHKA</t>
+  </si>
+  <si>
+    <t>AAVANI</t>
+  </si>
+  <si>
+    <t>BHAVYA</t>
+  </si>
+  <si>
+    <t>ASMI</t>
+  </si>
+  <si>
+    <t>CHAHAK</t>
+  </si>
+  <si>
+    <t>DEETYA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JANVI </t>
+  </si>
+  <si>
+    <t>KRATI</t>
+  </si>
+  <si>
+    <t>KANAK</t>
+  </si>
+  <si>
+    <t>RAHGVI</t>
+  </si>
+  <si>
+    <t>NANDINI</t>
+  </si>
+  <si>
+    <t>SAM</t>
+  </si>
+  <si>
+    <t>SAMRIDHI S</t>
+  </si>
+  <si>
+    <t>SAMRIDHI A</t>
+  </si>
+  <si>
+    <t>SURYA</t>
+  </si>
+  <si>
+    <t>UNATI</t>
+  </si>
+  <si>
+    <t>VRINDA</t>
+  </si>
+  <si>
+    <t>YASHASVI</t>
+  </si>
+  <si>
+    <t>on the floor</t>
+  </si>
+  <si>
+    <t>illegal ringtone</t>
+  </si>
+  <si>
+    <t>coutside</t>
+  </si>
+  <si>
+    <t>bad boy</t>
+  </si>
+  <si>
+    <t>police</t>
+  </si>
+  <si>
+    <t>Ramba Ho</t>
+  </si>
+  <si>
+    <t>tension</t>
+  </si>
+  <si>
+    <t>nightmare beats</t>
+  </si>
+  <si>
+    <t>fusion beats</t>
+  </si>
+  <si>
+    <t>do guna</t>
+  </si>
+  <si>
+    <t>kufar</t>
+  </si>
+  <si>
+    <t>hola amigo</t>
+  </si>
+  <si>
+    <t>local forecast</t>
+  </si>
+  <si>
+    <t>dracula</t>
+  </si>
+  <si>
+    <t>boyfriend</t>
+  </si>
+  <si>
+    <t>underground</t>
+  </si>
+  <si>
+    <t>real in rio x hot wings</t>
+  </si>
+  <si>
+    <t>way down we go</t>
+  </si>
+  <si>
+    <t>coook pardon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gozalo </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -328,6 +514,13 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -350,11 +543,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="20" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -587,15 +787,17 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C1" s="1"/>
     </row>
     <row r="2" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="B2" s="2"/>
+        <v>64</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>105</v>
+      </c>
       <c r="C2" s="2"/>
     </row>
     <row r="3" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -603,7 +805,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C3" s="2"/>
     </row>
@@ -612,37 +814,43 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C4" s="2"/>
     </row>
     <row r="5" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B5" s="2"/>
+        <v>54</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>96</v>
+      </c>
       <c r="C5" s="2"/>
     </row>
     <row r="6" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B6" s="2"/>
+        <v>70</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>106</v>
+      </c>
       <c r="C6" s="2"/>
     </row>
     <row r="7" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B7" s="2"/>
+        <v>44</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>87</v>
+      </c>
       <c r="C7" s="2"/>
     </row>
     <row r="8" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C8" s="2"/>
     </row>
@@ -655,116 +863,140 @@
     </row>
     <row r="10" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="2"/>
+        <v>15</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>133</v>
+      </c>
       <c r="C10" s="2"/>
     </row>
     <row r="11" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B11" s="2"/>
+        <v>22</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>86</v>
+      </c>
       <c r="C11" s="2"/>
     </row>
     <row r="12" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
     </row>
     <row r="13" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" s="2"/>
+        <v>23</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>137</v>
+      </c>
       <c r="C13" s="2"/>
     </row>
     <row r="14" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
     </row>
     <row r="15" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B15" s="2"/>
+        <v>55</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>142</v>
+      </c>
       <c r="C15" s="2"/>
     </row>
     <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B16" s="2"/>
+      <c r="B16" s="2" t="s">
+        <v>85</v>
+      </c>
       <c r="C16" s="2"/>
     </row>
     <row r="17" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B17" s="2"/>
+        <v>66</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>143</v>
+      </c>
       <c r="C17" s="2"/>
     </row>
     <row r="18" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="B18" s="2"/>
+        <v>56</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>94</v>
+      </c>
       <c r="C18" s="2"/>
     </row>
     <row r="19" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B19" s="2"/>
+        <v>46</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>95</v>
+      </c>
       <c r="C19" s="2"/>
     </row>
     <row r="20" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
     </row>
     <row r="21" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B21" s="2"/>
+        <v>18</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>145</v>
+      </c>
       <c r="C21" s="2"/>
     </row>
     <row r="22" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B22" s="2"/>
+        <v>24</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>93</v>
+      </c>
       <c r="C22" s="2"/>
     </row>
     <row r="23" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B23" s="2"/>
+        <v>47</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>138</v>
+      </c>
       <c r="C23" s="2"/>
     </row>
     <row r="24" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C24" s="2"/>
     </row>
     <row r="25" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B25" s="2"/>
+        <v>26</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>88</v>
+      </c>
       <c r="C25" s="2"/>
     </row>
     <row r="26" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -772,7 +1004,7 @@
         <v>5</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C26" s="2"/>
     </row>
@@ -781,55 +1013,65 @@
         <v>6</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C27" s="2"/>
     </row>
     <row r="28" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B28" s="2"/>
+        <v>67</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>139</v>
+      </c>
       <c r="C28" s="2"/>
     </row>
     <row r="29" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B29" s="2"/>
+        <v>27</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="C29" s="2"/>
     </row>
     <row r="30" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B30" s="2"/>
+        <v>32</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>140</v>
+      </c>
       <c r="C30" s="2"/>
     </row>
     <row r="31" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B31" s="2"/>
+        <v>59</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>146</v>
+      </c>
       <c r="C31" s="2"/>
     </row>
     <row r="32" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
     </row>
     <row r="33" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B33" s="2"/>
+        <v>57</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>104</v>
+      </c>
       <c r="C33" s="2"/>
     </row>
     <row r="34" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -852,37 +1094,39 @@
     </row>
     <row r="37" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B37" s="2"/>
+        <v>48</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>90</v>
+      </c>
       <c r="C37" s="2"/>
     </row>
     <row r="38" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A38" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
     </row>
     <row r="39" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A39" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
     </row>
     <row r="40" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A40" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="C40" s="2"/>
     </row>
     <row r="41" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A41" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -896,142 +1140,154 @@
     </row>
     <row r="43" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A43" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
     </row>
     <row r="44" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A44" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
     </row>
     <row r="45" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A45" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B45" s="2"/>
+        <v>33</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>103</v>
+      </c>
       <c r="C45" s="2"/>
     </row>
     <row r="46" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A46" s="2" t="s">
-        <v>12</v>
+        <v>91</v>
       </c>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
     </row>
     <row r="47" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A47" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
     </row>
     <row r="48" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A48" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>83</v>
+        <v>102</v>
       </c>
       <c r="C48" s="2"/>
     </row>
     <row r="49" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A49" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
     </row>
     <row r="50" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A50" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C50" s="2"/>
     </row>
     <row r="51" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A51" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
     </row>
     <row r="52" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A52" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B52" s="2"/>
+        <v>39</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="C52" s="2"/>
     </row>
     <row r="53" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A53" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B53" s="2"/>
+        <v>40</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>74</v>
+      </c>
       <c r="C53" s="2"/>
     </row>
     <row r="54" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A54" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B54" s="2"/>
+        <v>50</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>135</v>
+      </c>
       <c r="C54" s="2"/>
     </row>
     <row r="55" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A55" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B55" s="2"/>
+        <v>12</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>99</v>
+      </c>
       <c r="C55" s="2"/>
     </row>
     <row r="56" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A56" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
     </row>
     <row r="57" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A57" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B57" s="2"/>
+        <v>41</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>134</v>
+      </c>
       <c r="C57" s="2"/>
     </row>
     <row r="58" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A58" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
     </row>
     <row r="59" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A59" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
     </row>
     <row r="60" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A60" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C60" s="2"/>
     </row>
     <row r="61" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A61" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>76</v>
+        <v>100</v>
       </c>
       <c r="C61" s="2"/>
     </row>
@@ -1044,53 +1300,59 @@
     </row>
     <row r="63" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A63" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C63" s="2"/>
     </row>
     <row r="64" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A64" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
     </row>
     <row r="65" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A65" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B65" s="2"/>
+        <v>13</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>101</v>
+      </c>
       <c r="C65" s="2"/>
     </row>
     <row r="66" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A66" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B66" s="2"/>
+        <v>35</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>92</v>
+      </c>
       <c r="C66" s="2"/>
     </row>
     <row r="67" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A67" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
     </row>
     <row r="68" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A68" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B68" s="2"/>
       <c r="C68" s="2"/>
     </row>
     <row r="69" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A69" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="B69" s="2"/>
+        <v>61</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>141</v>
+      </c>
       <c r="C69" s="2"/>
     </row>
     <row r="70" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1098,76 +1360,198 @@
         <v>9</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C70" s="2"/>
     </row>
     <row r="71" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A71" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B71" s="2"/>
       <c r="C71" s="2"/>
     </row>
     <row r="72" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A72" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B72" s="2"/>
       <c r="C72" s="2"/>
     </row>
     <row r="73" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A73" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="C73" s="2"/>
     </row>
     <row r="74" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="C74" s="2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="76" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="77" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="78" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="79" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="80" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="81" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="82" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="83" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="84" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="85" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="86" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="87" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="88" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="89" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="90" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="91" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="92" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="93" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="94" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="95" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="96" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="97" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="98" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="99" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="100" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="101" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="102" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="103" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="104" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="105" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="106" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="107" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="108" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="109" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="110" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="111" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="112" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+        <v>71</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A75" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A76" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A77" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A78" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A79" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A80" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A81" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B81" s="6" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A82" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B82" s="5"/>
+    </row>
+    <row r="83" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A83" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A84" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A85" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A86" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A87" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B87" s="6" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A88" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B88" s="5"/>
+    </row>
+    <row r="89" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A89" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B89" s="6" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A90" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B90" s="5"/>
+    </row>
+    <row r="91" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A91" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B91" s="6" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A92" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B92" s="5"/>
+    </row>
+    <row r="93" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A93" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B93" s="6" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A94" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B94" s="5"/>
+    </row>
+    <row r="95" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A95" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A96" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A97" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A98" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="100" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="101" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="102" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="103" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="104" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="105" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="106" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="107" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="108" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="109" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="110" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="111" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="112" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="113" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="114" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="115" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
@@ -2060,6 +2444,13 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:A73">
     <sortCondition ref="A2:A73"/>
   </sortState>
+  <mergeCells count="5">
+    <mergeCell ref="B91:B92"/>
+    <mergeCell ref="B87:B88"/>
+    <mergeCell ref="B89:B90"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="B93:B94"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>